<commit_message>
removed images and extra results
</commit_message>
<xml_diff>
--- a/results/results.xlsx
+++ b/results/results.xlsx
@@ -513,25 +513,25 @@
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>128.1</v>
+        <v>4.9</v>
       </c>
       <c r="D2" t="n">
-        <v>177.1</v>
+        <v>5.1</v>
       </c>
       <c r="E2" t="n">
-        <v>237</v>
+        <v>5.3</v>
       </c>
       <c r="F2" t="n">
-        <v>258.7</v>
+        <v>12.1</v>
       </c>
       <c r="G2" t="n">
-        <v>284.4</v>
+        <v>43.7</v>
       </c>
       <c r="H2" t="n">
-        <v>808.6</v>
+        <v>195.7</v>
       </c>
       <c r="I2" t="n">
-        <v>808.6</v>
+        <v>266.5</v>
       </c>
     </row>
     <row r="3">
@@ -544,25 +544,25 @@
         <v>2</v>
       </c>
       <c r="C3" t="n">
-        <v>154.7</v>
+        <v>4.9</v>
       </c>
       <c r="D3" t="n">
-        <v>215.5</v>
+        <v>5.1</v>
       </c>
       <c r="E3" t="n">
-        <v>246.2</v>
+        <v>5.4</v>
       </c>
       <c r="F3" t="n">
-        <v>263.2</v>
+        <v>9.6</v>
       </c>
       <c r="G3" t="n">
-        <v>288.4</v>
+        <v>43.4</v>
       </c>
       <c r="H3" t="n">
-        <v>398.2</v>
+        <v>195.7</v>
       </c>
       <c r="I3" t="n">
-        <v>398.2</v>
+        <v>243.5</v>
       </c>
     </row>
     <row r="4">
@@ -575,25 +575,25 @@
         <v>3</v>
       </c>
       <c r="C4" t="n">
-        <v>154.2</v>
+        <v>5</v>
       </c>
       <c r="D4" t="n">
-        <v>203</v>
+        <v>5.2</v>
       </c>
       <c r="E4" t="n">
-        <v>235.8</v>
+        <v>5.5</v>
       </c>
       <c r="F4" t="n">
-        <v>259.8</v>
+        <v>10.6</v>
       </c>
       <c r="G4" t="n">
-        <v>296.7</v>
+        <v>41.8</v>
       </c>
       <c r="H4" t="n">
-        <v>473.2</v>
+        <v>195.3</v>
       </c>
       <c r="I4" t="n">
-        <v>473.2</v>
+        <v>249</v>
       </c>
     </row>
     <row r="5">
@@ -606,25 +606,25 @@
         <v>4</v>
       </c>
       <c r="C5" t="n">
-        <v>133.8</v>
+        <v>5</v>
       </c>
       <c r="D5" t="n">
-        <v>204.1</v>
+        <v>5.1</v>
       </c>
       <c r="E5" t="n">
-        <v>244.4</v>
+        <v>5.3</v>
       </c>
       <c r="F5" t="n">
-        <v>258.7</v>
+        <v>11.4</v>
       </c>
       <c r="G5" t="n">
-        <v>307.5</v>
+        <v>45</v>
       </c>
       <c r="H5" t="n">
-        <v>473.6</v>
+        <v>200.6</v>
       </c>
       <c r="I5" t="n">
-        <v>473.6</v>
+        <v>243.7</v>
       </c>
     </row>
     <row r="6">
@@ -637,25 +637,25 @@
         <v>5</v>
       </c>
       <c r="C6" t="n">
-        <v>155</v>
+        <v>5</v>
       </c>
       <c r="D6" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="E6" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="F6" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="G6" t="n">
+        <v>45.9</v>
+      </c>
+      <c r="H6" t="n">
         <v>201.4</v>
       </c>
-      <c r="E6" t="n">
-        <v>238.4</v>
-      </c>
-      <c r="F6" t="n">
-        <v>257.5</v>
-      </c>
-      <c r="G6" t="n">
-        <v>296.5</v>
-      </c>
-      <c r="H6" t="n">
-        <v>714</v>
-      </c>
       <c r="I6" t="n">
-        <v>714</v>
+        <v>260.8</v>
       </c>
     </row>
     <row r="7">
@@ -668,25 +668,25 @@
         <v>6</v>
       </c>
       <c r="C7" t="n">
-        <v>164.7</v>
+        <v>5</v>
       </c>
       <c r="D7" t="n">
-        <v>207.6</v>
+        <v>5.1</v>
       </c>
       <c r="E7" t="n">
-        <v>245.2</v>
+        <v>5.4</v>
       </c>
       <c r="F7" t="n">
-        <v>261.6</v>
+        <v>10.4</v>
       </c>
       <c r="G7" t="n">
-        <v>316.2</v>
+        <v>50.4</v>
       </c>
       <c r="H7" t="n">
-        <v>539.8</v>
+        <v>203.2</v>
       </c>
       <c r="I7" t="n">
-        <v>539.8</v>
+        <v>390.5</v>
       </c>
     </row>
     <row r="8">
@@ -699,25 +699,25 @@
         <v>7</v>
       </c>
       <c r="C8" t="n">
-        <v>135.3</v>
+        <v>4.9</v>
       </c>
       <c r="D8" t="n">
-        <v>215.1</v>
+        <v>5.1</v>
       </c>
       <c r="E8" t="n">
-        <v>244.3</v>
+        <v>5.3</v>
       </c>
       <c r="F8" t="n">
-        <v>279</v>
+        <v>11</v>
       </c>
       <c r="G8" t="n">
-        <v>325.1</v>
+        <v>46.5</v>
       </c>
       <c r="H8" t="n">
-        <v>1725.4</v>
+        <v>198.2</v>
       </c>
       <c r="I8" t="n">
-        <v>1725.4</v>
+        <v>247.3</v>
       </c>
     </row>
     <row r="9">
@@ -730,25 +730,25 @@
         <v>8</v>
       </c>
       <c r="C9" t="n">
-        <v>139.1</v>
+        <v>5</v>
       </c>
       <c r="D9" t="n">
-        <v>215.7</v>
+        <v>5.1</v>
       </c>
       <c r="E9" t="n">
-        <v>240.2</v>
+        <v>5.3</v>
       </c>
       <c r="F9" t="n">
-        <v>258.8</v>
+        <v>10.4</v>
       </c>
       <c r="G9" t="n">
-        <v>291.3</v>
+        <v>45.8</v>
       </c>
       <c r="H9" t="n">
-        <v>729.3</v>
+        <v>204</v>
       </c>
       <c r="I9" t="n">
-        <v>729.3</v>
+        <v>257.4</v>
       </c>
     </row>
     <row r="10">
@@ -761,25 +761,25 @@
         <v>9</v>
       </c>
       <c r="C10" t="n">
-        <v>164.6</v>
+        <v>4.9</v>
       </c>
       <c r="D10" t="n">
-        <v>211.3</v>
+        <v>5.1</v>
       </c>
       <c r="E10" t="n">
-        <v>243.2</v>
+        <v>5.3</v>
       </c>
       <c r="F10" t="n">
-        <v>261.4</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="G10" t="n">
-        <v>296.8</v>
+        <v>45.6</v>
       </c>
       <c r="H10" t="n">
-        <v>586.9</v>
+        <v>198.5</v>
       </c>
       <c r="I10" t="n">
-        <v>586.9</v>
+        <v>267.4</v>
       </c>
     </row>
     <row r="11">
@@ -792,25 +792,25 @@
         <v>10</v>
       </c>
       <c r="C11" t="n">
-        <v>163.5</v>
+        <v>5</v>
       </c>
       <c r="D11" t="n">
-        <v>215.9</v>
+        <v>5.1</v>
       </c>
       <c r="E11" t="n">
-        <v>244.2</v>
+        <v>5.4</v>
       </c>
       <c r="F11" t="n">
-        <v>261.5</v>
+        <v>12.8</v>
       </c>
       <c r="G11" t="n">
-        <v>295.8</v>
+        <v>49</v>
       </c>
       <c r="H11" t="n">
-        <v>492.8</v>
+        <v>201.5</v>
       </c>
       <c r="I11" t="n">
-        <v>492.8</v>
+        <v>287.2</v>
       </c>
     </row>
     <row r="12">
@@ -825,25 +825,25 @@
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>149.3</v>
+        <v>4.96</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>206.67</v>
+        <v>5.12</v>
       </c>
       <c r="E12" s="2" t="n">
-        <v>241.89</v>
+        <v>5.37</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>262.02</v>
+        <v>10.96</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>299.87</v>
+        <v>45.71</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>694.1799999999999</v>
+        <v>199.41</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>694.1799999999999</v>
+        <v>271.33</v>
       </c>
     </row>
     <row r="13">
@@ -858,25 +858,25 @@
         </is>
       </c>
       <c r="C13" s="3" t="n">
-        <v>13.937</v>
+        <v>0.052</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>11.834</v>
+        <v>0.042</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>3.723</v>
+        <v>0.082</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>6.221</v>
+        <v>1.007</v>
       </c>
       <c r="G13" s="3" t="n">
-        <v>12.707</v>
+        <v>2.553</v>
       </c>
       <c r="H13" s="3" t="n">
-        <v>385.735</v>
+        <v>3.195</v>
       </c>
       <c r="I13" s="3" t="n">
-        <v>385.735</v>
+        <v>43.984</v>
       </c>
     </row>
     <row r="15">
@@ -889,25 +889,25 @@
         <v>1</v>
       </c>
       <c r="C15" t="n">
-        <v>164.6</v>
+        <v>5</v>
       </c>
       <c r="D15" t="n">
-        <v>205.7</v>
+        <v>5.2</v>
       </c>
       <c r="E15" t="n">
-        <v>242.7</v>
+        <v>5.5</v>
       </c>
       <c r="F15" t="n">
-        <v>261</v>
+        <v>11.6</v>
       </c>
       <c r="G15" t="n">
-        <v>292.5</v>
+        <v>46.5</v>
       </c>
       <c r="H15" t="n">
-        <v>914.7</v>
+        <v>197.8</v>
       </c>
       <c r="I15" t="n">
-        <v>914.7</v>
+        <v>281.1</v>
       </c>
     </row>
     <row r="16">
@@ -920,25 +920,25 @@
         <v>2</v>
       </c>
       <c r="C16" t="n">
-        <v>138.2</v>
+        <v>4.9</v>
       </c>
       <c r="D16" t="n">
-        <v>195.8</v>
+        <v>5.1</v>
       </c>
       <c r="E16" t="n">
-        <v>223.7</v>
+        <v>5.4</v>
       </c>
       <c r="F16" t="n">
-        <v>239.3</v>
+        <v>11.8</v>
       </c>
       <c r="G16" t="n">
-        <v>274.6</v>
+        <v>47.2</v>
       </c>
       <c r="H16" t="n">
-        <v>904.8</v>
+        <v>202.5</v>
       </c>
       <c r="I16" t="n">
-        <v>904.8</v>
+        <v>265.9</v>
       </c>
     </row>
     <row r="17">
@@ -951,25 +951,25 @@
         <v>3</v>
       </c>
       <c r="C17" t="n">
-        <v>157.2</v>
+        <v>5</v>
       </c>
       <c r="D17" t="n">
-        <v>201.2</v>
+        <v>5.1</v>
       </c>
       <c r="E17" t="n">
-        <v>223.8</v>
+        <v>5.4</v>
       </c>
       <c r="F17" t="n">
-        <v>259.6</v>
+        <v>10.9</v>
       </c>
       <c r="G17" t="n">
-        <v>285.1</v>
+        <v>48.6</v>
       </c>
       <c r="H17" t="n">
-        <v>598.6</v>
+        <v>197.2</v>
       </c>
       <c r="I17" t="n">
-        <v>598.6</v>
+        <v>273.4</v>
       </c>
     </row>
     <row r="18">
@@ -982,25 +982,25 @@
         <v>4</v>
       </c>
       <c r="C18" t="n">
-        <v>179</v>
+        <v>5.1</v>
       </c>
       <c r="D18" t="n">
-        <v>210.6</v>
+        <v>5.2</v>
       </c>
       <c r="E18" t="n">
-        <v>232.7</v>
+        <v>5.5</v>
       </c>
       <c r="F18" t="n">
-        <v>257.9</v>
+        <v>12.7</v>
       </c>
       <c r="G18" t="n">
+        <v>39.7</v>
+      </c>
+      <c r="H18" t="n">
+        <v>200.8</v>
+      </c>
+      <c r="I18" t="n">
         <v>284.2</v>
-      </c>
-      <c r="H18" t="n">
-        <v>566.9</v>
-      </c>
-      <c r="I18" t="n">
-        <v>566.9</v>
       </c>
     </row>
     <row r="19">
@@ -1013,25 +1013,25 @@
         <v>5</v>
       </c>
       <c r="C19" t="n">
-        <v>154.6</v>
+        <v>4.8</v>
       </c>
       <c r="D19" t="n">
-        <v>201.2</v>
+        <v>4.9</v>
       </c>
       <c r="E19" t="n">
-        <v>222.6</v>
+        <v>5.2</v>
       </c>
       <c r="F19" t="n">
-        <v>256.6</v>
+        <v>10</v>
       </c>
       <c r="G19" t="n">
-        <v>274.9</v>
+        <v>46.7</v>
       </c>
       <c r="H19" t="n">
-        <v>425.6</v>
+        <v>201.1</v>
       </c>
       <c r="I19" t="n">
-        <v>425.6</v>
+        <v>305.3</v>
       </c>
     </row>
     <row r="20">
@@ -1044,25 +1044,25 @@
         <v>6</v>
       </c>
       <c r="C20" t="n">
-        <v>139.7</v>
+        <v>5.1</v>
       </c>
       <c r="D20" t="n">
-        <v>197.1</v>
+        <v>5.3</v>
       </c>
       <c r="E20" t="n">
-        <v>229.2</v>
+        <v>5.6</v>
       </c>
       <c r="F20" t="n">
-        <v>258.2</v>
+        <v>11.7</v>
       </c>
       <c r="G20" t="n">
-        <v>289.4</v>
+        <v>44.3</v>
       </c>
       <c r="H20" t="n">
-        <v>698.3</v>
+        <v>199.2</v>
       </c>
       <c r="I20" t="n">
-        <v>698.3</v>
+        <v>251</v>
       </c>
     </row>
     <row r="21">
@@ -1075,25 +1075,25 @@
         <v>7</v>
       </c>
       <c r="C21" t="n">
-        <v>173.9</v>
+        <v>5.1</v>
       </c>
       <c r="D21" t="n">
-        <v>208.7</v>
+        <v>5.3</v>
       </c>
       <c r="E21" t="n">
-        <v>234.5</v>
+        <v>5.6</v>
       </c>
       <c r="F21" t="n">
-        <v>260</v>
+        <v>12</v>
       </c>
       <c r="G21" t="n">
-        <v>288.8</v>
+        <v>44.5</v>
       </c>
       <c r="H21" t="n">
-        <v>728.5</v>
+        <v>198.8</v>
       </c>
       <c r="I21" t="n">
-        <v>728.5</v>
+        <v>251.4</v>
       </c>
     </row>
     <row r="22">
@@ -1106,25 +1106,25 @@
         <v>8</v>
       </c>
       <c r="C22" t="n">
-        <v>155.8</v>
+        <v>4.8</v>
       </c>
       <c r="D22" t="n">
-        <v>200.4</v>
+        <v>4.9</v>
       </c>
       <c r="E22" t="n">
-        <v>238.9</v>
+        <v>5.2</v>
       </c>
       <c r="F22" t="n">
-        <v>258.1</v>
+        <v>10.2</v>
       </c>
       <c r="G22" t="n">
-        <v>282.3</v>
+        <v>46.8</v>
       </c>
       <c r="H22" t="n">
-        <v>562.8</v>
+        <v>194.8</v>
       </c>
       <c r="I22" t="n">
-        <v>562.8</v>
+        <v>244.2</v>
       </c>
     </row>
     <row r="23">
@@ -1137,25 +1137,25 @@
         <v>9</v>
       </c>
       <c r="C23" t="n">
-        <v>170.8</v>
+        <v>5</v>
       </c>
       <c r="D23" t="n">
-        <v>210.7</v>
+        <v>5.2</v>
       </c>
       <c r="E23" t="n">
-        <v>234.6</v>
+        <v>5.4</v>
       </c>
       <c r="F23" t="n">
-        <v>260</v>
+        <v>10.5</v>
       </c>
       <c r="G23" t="n">
-        <v>291.5</v>
+        <v>49.1</v>
       </c>
       <c r="H23" t="n">
-        <v>613</v>
+        <v>199.3</v>
       </c>
       <c r="I23" t="n">
-        <v>613</v>
+        <v>259.8</v>
       </c>
     </row>
     <row r="24">
@@ -1168,25 +1168,25 @@
         <v>10</v>
       </c>
       <c r="C24" t="n">
-        <v>152</v>
+        <v>5</v>
       </c>
       <c r="D24" t="n">
-        <v>205.3</v>
+        <v>5.2</v>
       </c>
       <c r="E24" t="n">
-        <v>224.1</v>
+        <v>5.6</v>
       </c>
       <c r="F24" t="n">
-        <v>244.8</v>
+        <v>12.8</v>
       </c>
       <c r="G24" t="n">
-        <v>276.1</v>
+        <v>48.4</v>
       </c>
       <c r="H24" t="n">
-        <v>1027.5</v>
+        <v>200.7</v>
       </c>
       <c r="I24" t="n">
-        <v>1027.5</v>
+        <v>313.7</v>
       </c>
     </row>
     <row r="25">
@@ -1201,25 +1201,25 @@
         </is>
       </c>
       <c r="C25" s="2" t="n">
-        <v>158.58</v>
+        <v>4.98</v>
       </c>
       <c r="D25" s="2" t="n">
-        <v>203.67</v>
+        <v>5.14</v>
       </c>
       <c r="E25" s="2" t="n">
-        <v>230.68</v>
+        <v>5.44</v>
       </c>
       <c r="F25" s="2" t="n">
-        <v>255.55</v>
+        <v>11.42</v>
       </c>
       <c r="G25" s="2" t="n">
-        <v>283.94</v>
+        <v>46.18</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>704.0700000000001</v>
+        <v>199.22</v>
       </c>
       <c r="I25" s="2" t="n">
-        <v>704.0700000000001</v>
+        <v>273</v>
       </c>
     </row>
     <row r="26">
@@ -1234,25 +1234,25 @@
         </is>
       </c>
       <c r="C26" s="3" t="n">
-        <v>13.654</v>
+        <v>0.114</v>
       </c>
       <c r="D26" s="3" t="n">
-        <v>5.349</v>
+        <v>0.143</v>
       </c>
       <c r="E26" s="3" t="n">
-        <v>7.094</v>
+        <v>0.151</v>
       </c>
       <c r="F26" s="3" t="n">
-        <v>7.345</v>
+        <v>0.986</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>6.818</v>
+        <v>2.778</v>
       </c>
       <c r="H26" s="3" t="n">
-        <v>190.214</v>
+        <v>2.231</v>
       </c>
       <c r="I26" s="3" t="n">
-        <v>190.214</v>
+        <v>23.323</v>
       </c>
     </row>
     <row r="28">
@@ -1265,25 +1265,25 @@
         <v>1</v>
       </c>
       <c r="C28" t="n">
-        <v>142.2</v>
+        <v>5.2</v>
       </c>
       <c r="D28" t="n">
-        <v>212.3</v>
+        <v>5.6</v>
       </c>
       <c r="E28" t="n">
-        <v>238.7</v>
+        <v>9</v>
       </c>
       <c r="F28" t="n">
-        <v>260</v>
+        <v>21.5</v>
       </c>
       <c r="G28" t="n">
-        <v>316.4</v>
+        <v>45.2</v>
       </c>
       <c r="H28" t="n">
-        <v>1308.2</v>
+        <v>203.8</v>
       </c>
       <c r="I28" t="n">
-        <v>1308.2</v>
+        <v>432.3</v>
       </c>
     </row>
     <row r="29">
@@ -1296,25 +1296,25 @@
         <v>2</v>
       </c>
       <c r="C29" t="n">
-        <v>127.2</v>
+        <v>5.1</v>
       </c>
       <c r="D29" t="n">
-        <v>214</v>
+        <v>5.5</v>
       </c>
       <c r="E29" t="n">
-        <v>238.4</v>
+        <v>9</v>
       </c>
       <c r="F29" t="n">
-        <v>255.3</v>
+        <v>21.2</v>
       </c>
       <c r="G29" t="n">
-        <v>292.8</v>
+        <v>45.4</v>
       </c>
       <c r="H29" t="n">
-        <v>574.5</v>
+        <v>205.9</v>
       </c>
       <c r="I29" t="n">
-        <v>574.5</v>
+        <v>384.7</v>
       </c>
     </row>
     <row r="30">
@@ -1327,25 +1327,25 @@
         <v>3</v>
       </c>
       <c r="C30" t="n">
-        <v>124.1</v>
+        <v>5</v>
       </c>
       <c r="D30" t="n">
-        <v>216.8</v>
+        <v>5.5</v>
       </c>
       <c r="E30" t="n">
-        <v>248.1</v>
+        <v>9.1</v>
       </c>
       <c r="F30" t="n">
-        <v>261.3</v>
+        <v>21.7</v>
       </c>
       <c r="G30" t="n">
-        <v>349.7</v>
+        <v>46.4</v>
       </c>
       <c r="H30" t="n">
-        <v>527.2</v>
+        <v>204.1</v>
       </c>
       <c r="I30" t="n">
-        <v>527.2</v>
+        <v>287.6</v>
       </c>
     </row>
     <row r="31">
@@ -1358,25 +1358,25 @@
         <v>4</v>
       </c>
       <c r="C31" t="n">
-        <v>137.4</v>
+        <v>5.1</v>
       </c>
       <c r="D31" t="n">
-        <v>219.5</v>
+        <v>5.6</v>
       </c>
       <c r="E31" t="n">
-        <v>254.1</v>
+        <v>8.9</v>
       </c>
       <c r="F31" t="n">
-        <v>275.3</v>
+        <v>21.7</v>
       </c>
       <c r="G31" t="n">
-        <v>315.7</v>
+        <v>44.4</v>
       </c>
       <c r="H31" t="n">
-        <v>686.3</v>
+        <v>202.1</v>
       </c>
       <c r="I31" t="n">
-        <v>686.3</v>
+        <v>394.1</v>
       </c>
     </row>
     <row r="32">
@@ -1389,25 +1389,25 @@
         <v>5</v>
       </c>
       <c r="C32" t="n">
-        <v>134.7</v>
+        <v>5.1</v>
       </c>
       <c r="D32" t="n">
-        <v>200.6</v>
+        <v>5.6</v>
       </c>
       <c r="E32" t="n">
-        <v>244.5</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="F32" t="n">
-        <v>267.1</v>
+        <v>21.2</v>
       </c>
       <c r="G32" t="n">
-        <v>359.1</v>
+        <v>44.2</v>
       </c>
       <c r="H32" t="n">
-        <v>846.1</v>
+        <v>205.1</v>
       </c>
       <c r="I32" t="n">
-        <v>846.1</v>
+        <v>374.1</v>
       </c>
     </row>
     <row r="33">
@@ -1420,25 +1420,25 @@
         <v>6</v>
       </c>
       <c r="C33" t="n">
-        <v>134.4</v>
+        <v>5.1</v>
       </c>
       <c r="D33" t="n">
-        <v>220.6</v>
+        <v>5.6</v>
       </c>
       <c r="E33" t="n">
-        <v>250</v>
+        <v>8.9</v>
       </c>
       <c r="F33" t="n">
-        <v>274.3</v>
+        <v>21</v>
       </c>
       <c r="G33" t="n">
-        <v>355.2</v>
+        <v>44.6</v>
       </c>
       <c r="H33" t="n">
-        <v>972.1</v>
+        <v>207.4</v>
       </c>
       <c r="I33" t="n">
-        <v>972.1</v>
+        <v>292.9</v>
       </c>
     </row>
     <row r="34">
@@ -1451,25 +1451,25 @@
         <v>7</v>
       </c>
       <c r="C34" t="n">
-        <v>130.1</v>
+        <v>5.2</v>
       </c>
       <c r="D34" t="n">
-        <v>209.4</v>
+        <v>5.7</v>
       </c>
       <c r="E34" t="n">
-        <v>240.1</v>
+        <v>9.4</v>
       </c>
       <c r="F34" t="n">
-        <v>263.7</v>
+        <v>21.4</v>
       </c>
       <c r="G34" t="n">
-        <v>298</v>
+        <v>44.3</v>
       </c>
       <c r="H34" t="n">
-        <v>767.2</v>
+        <v>205.8</v>
       </c>
       <c r="I34" t="n">
-        <v>767.2</v>
+        <v>282.5</v>
       </c>
     </row>
     <row r="35">
@@ -1482,25 +1482,25 @@
         <v>8</v>
       </c>
       <c r="C35" t="n">
-        <v>135.6</v>
+        <v>5.1</v>
       </c>
       <c r="D35" t="n">
-        <v>222.6</v>
+        <v>5.7</v>
       </c>
       <c r="E35" t="n">
-        <v>248.7</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="F35" t="n">
-        <v>274.6</v>
+        <v>21.3</v>
       </c>
       <c r="G35" t="n">
-        <v>345.5</v>
+        <v>45.1</v>
       </c>
       <c r="H35" t="n">
-        <v>1217.3</v>
+        <v>204.3</v>
       </c>
       <c r="I35" t="n">
-        <v>1217.3</v>
+        <v>293.1</v>
       </c>
     </row>
     <row r="36">
@@ -1513,25 +1513,25 @@
         <v>9</v>
       </c>
       <c r="C36" t="n">
-        <v>146.3</v>
+        <v>5.1</v>
       </c>
       <c r="D36" t="n">
-        <v>200</v>
+        <v>5.6</v>
       </c>
       <c r="E36" t="n">
-        <v>252.5</v>
+        <v>8.9</v>
       </c>
       <c r="F36" t="n">
-        <v>261.5</v>
+        <v>21.3</v>
       </c>
       <c r="G36" t="n">
-        <v>328.2</v>
+        <v>44</v>
       </c>
       <c r="H36" t="n">
-        <v>653.7</v>
+        <v>204.1</v>
       </c>
       <c r="I36" t="n">
-        <v>653.7</v>
+        <v>272.3</v>
       </c>
     </row>
     <row r="37">
@@ -1544,25 +1544,25 @@
         <v>10</v>
       </c>
       <c r="C37" t="n">
-        <v>129.4</v>
+        <v>5.1</v>
       </c>
       <c r="D37" t="n">
-        <v>212</v>
+        <v>5.6</v>
       </c>
       <c r="E37" t="n">
-        <v>242.6</v>
+        <v>9.1</v>
       </c>
       <c r="F37" t="n">
-        <v>263.4</v>
+        <v>21.4</v>
       </c>
       <c r="G37" t="n">
-        <v>284.4</v>
+        <v>41.6</v>
       </c>
       <c r="H37" t="n">
-        <v>809.3</v>
+        <v>203.8</v>
       </c>
       <c r="I37" t="n">
-        <v>809.3</v>
+        <v>297.9</v>
       </c>
     </row>
     <row r="38">
@@ -1577,25 +1577,25 @@
         </is>
       </c>
       <c r="C38" s="2" t="n">
-        <v>134.14</v>
+        <v>5.11</v>
       </c>
       <c r="D38" s="2" t="n">
-        <v>212.78</v>
+        <v>5.6</v>
       </c>
       <c r="E38" s="2" t="n">
-        <v>245.77</v>
+        <v>9.130000000000001</v>
       </c>
       <c r="F38" s="2" t="n">
-        <v>265.65</v>
+        <v>21.37</v>
       </c>
       <c r="G38" s="2" t="n">
-        <v>324.5</v>
+        <v>44.52</v>
       </c>
       <c r="H38" s="2" t="n">
-        <v>836.1900000000001</v>
+        <v>204.64</v>
       </c>
       <c r="I38" s="2" t="n">
-        <v>836.1900000000001</v>
+        <v>331.15</v>
       </c>
     </row>
     <row r="39">
@@ -1610,25 +1610,25 @@
         </is>
       </c>
       <c r="C39" s="3" t="n">
-        <v>6.78</v>
+        <v>0.057</v>
       </c>
       <c r="D39" s="3" t="n">
-        <v>7.777</v>
+        <v>0.067</v>
       </c>
       <c r="E39" s="3" t="n">
-        <v>5.722</v>
+        <v>0.283</v>
       </c>
       <c r="F39" s="3" t="n">
-        <v>6.946</v>
+        <v>0.221</v>
       </c>
       <c r="G39" s="3" t="n">
-        <v>27.259</v>
+        <v>1.251</v>
       </c>
       <c r="H39" s="3" t="n">
-        <v>260.729</v>
+        <v>1.465</v>
       </c>
       <c r="I39" s="3" t="n">
-        <v>260.729</v>
+        <v>58.357</v>
       </c>
     </row>
     <row r="41">
@@ -1641,25 +1641,25 @@
         <v>1</v>
       </c>
       <c r="C41" t="n">
-        <v>156.9</v>
+        <v>5.1</v>
       </c>
       <c r="D41" t="n">
-        <v>223.9</v>
+        <v>5.2</v>
       </c>
       <c r="E41" t="n">
-        <v>241.4</v>
+        <v>5.5</v>
       </c>
       <c r="F41" t="n">
-        <v>251.5</v>
+        <v>10.3</v>
       </c>
       <c r="G41" t="n">
-        <v>265.8</v>
+        <v>45.7</v>
       </c>
       <c r="H41" t="n">
-        <v>875.4</v>
+        <v>202.5</v>
       </c>
       <c r="I41" t="n">
-        <v>875.4</v>
+        <v>301.6</v>
       </c>
     </row>
     <row r="42">
@@ -1672,25 +1672,25 @@
         <v>2</v>
       </c>
       <c r="C42" t="n">
-        <v>158.1</v>
+        <v>5.3</v>
       </c>
       <c r="D42" t="n">
-        <v>214.6</v>
+        <v>5.5</v>
       </c>
       <c r="E42" t="n">
-        <v>252.8</v>
+        <v>5.8</v>
       </c>
       <c r="F42" t="n">
-        <v>280.7</v>
+        <v>9.9</v>
       </c>
       <c r="G42" t="n">
-        <v>330.7</v>
+        <v>43.9</v>
       </c>
       <c r="H42" t="n">
-        <v>598</v>
+        <v>192.9</v>
       </c>
       <c r="I42" t="n">
-        <v>598</v>
+        <v>252</v>
       </c>
     </row>
     <row r="43">
@@ -1703,25 +1703,25 @@
         <v>3</v>
       </c>
       <c r="C43" t="n">
-        <v>125.6</v>
+        <v>5</v>
       </c>
       <c r="D43" t="n">
-        <v>204.2</v>
+        <v>5.1</v>
       </c>
       <c r="E43" t="n">
-        <v>230.1</v>
+        <v>5.3</v>
       </c>
       <c r="F43" t="n">
-        <v>252.3</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="G43" t="n">
-        <v>268.9</v>
+        <v>45.4</v>
       </c>
       <c r="H43" t="n">
-        <v>674.5</v>
+        <v>196.8</v>
       </c>
       <c r="I43" t="n">
-        <v>674.5</v>
+        <v>280.3</v>
       </c>
     </row>
     <row r="44">
@@ -1734,25 +1734,25 @@
         <v>4</v>
       </c>
       <c r="C44" t="n">
-        <v>129.3</v>
+        <v>5</v>
       </c>
       <c r="D44" t="n">
-        <v>196.9</v>
+        <v>5.1</v>
       </c>
       <c r="E44" t="n">
-        <v>232.3</v>
+        <v>5.3</v>
       </c>
       <c r="F44" t="n">
-        <v>258.2</v>
+        <v>10.2</v>
       </c>
       <c r="G44" t="n">
-        <v>285.3</v>
+        <v>43.9</v>
       </c>
       <c r="H44" t="n">
-        <v>372.3</v>
+        <v>195.3</v>
       </c>
       <c r="I44" t="n">
-        <v>372.3</v>
+        <v>284.5</v>
       </c>
     </row>
     <row r="45">
@@ -1765,25 +1765,25 @@
         <v>5</v>
       </c>
       <c r="C45" t="n">
-        <v>154</v>
+        <v>4.9</v>
       </c>
       <c r="D45" t="n">
-        <v>203.4</v>
+        <v>5</v>
       </c>
       <c r="E45" t="n">
-        <v>243.8</v>
+        <v>5.3</v>
       </c>
       <c r="F45" t="n">
-        <v>256.8</v>
+        <v>10.7</v>
       </c>
       <c r="G45" t="n">
-        <v>319.1</v>
+        <v>46</v>
       </c>
       <c r="H45" t="n">
-        <v>640.7</v>
+        <v>198.4</v>
       </c>
       <c r="I45" t="n">
-        <v>640.7</v>
+        <v>243</v>
       </c>
     </row>
     <row r="46">
@@ -1796,25 +1796,25 @@
         <v>6</v>
       </c>
       <c r="C46" t="n">
-        <v>168.9</v>
+        <v>4.9</v>
       </c>
       <c r="D46" t="n">
-        <v>213.2</v>
+        <v>5.1</v>
       </c>
       <c r="E46" t="n">
-        <v>238</v>
+        <v>5.3</v>
       </c>
       <c r="F46" t="n">
-        <v>263.6</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="G46" t="n">
-        <v>299.9</v>
+        <v>44.7</v>
       </c>
       <c r="H46" t="n">
-        <v>514.5</v>
+        <v>200</v>
       </c>
       <c r="I46" t="n">
-        <v>514.5</v>
+        <v>234.5</v>
       </c>
     </row>
     <row r="47">
@@ -1827,25 +1827,25 @@
         <v>7</v>
       </c>
       <c r="C47" t="n">
-        <v>174.7</v>
+        <v>4.8</v>
       </c>
       <c r="D47" t="n">
-        <v>216.7</v>
+        <v>5</v>
       </c>
       <c r="E47" t="n">
-        <v>249.6</v>
+        <v>5.2</v>
       </c>
       <c r="F47" t="n">
-        <v>261.7</v>
+        <v>10.8</v>
       </c>
       <c r="G47" t="n">
-        <v>293.7</v>
+        <v>40.9</v>
       </c>
       <c r="H47" t="n">
-        <v>416.5</v>
+        <v>196.8</v>
       </c>
       <c r="I47" t="n">
-        <v>416.5</v>
+        <v>278.3</v>
       </c>
     </row>
     <row r="48">
@@ -1858,25 +1858,25 @@
         <v>8</v>
       </c>
       <c r="C48" t="n">
-        <v>136.7</v>
+        <v>4.9</v>
       </c>
       <c r="D48" t="n">
-        <v>203.6</v>
+        <v>5.2</v>
       </c>
       <c r="E48" t="n">
-        <v>225.3</v>
+        <v>5.6</v>
       </c>
       <c r="F48" t="n">
-        <v>253</v>
+        <v>11.2</v>
       </c>
       <c r="G48" t="n">
-        <v>274.7</v>
+        <v>48</v>
       </c>
       <c r="H48" t="n">
-        <v>751.3</v>
+        <v>197</v>
       </c>
       <c r="I48" t="n">
-        <v>751.3</v>
+        <v>245.7</v>
       </c>
     </row>
     <row r="49">
@@ -1889,25 +1889,25 @@
         <v>9</v>
       </c>
       <c r="C49" t="n">
-        <v>148.7</v>
+        <v>5</v>
       </c>
       <c r="D49" t="n">
-        <v>196.8</v>
+        <v>5.1</v>
       </c>
       <c r="E49" t="n">
-        <v>234.9</v>
+        <v>5.3</v>
       </c>
       <c r="F49" t="n">
-        <v>252.9</v>
+        <v>10.4</v>
       </c>
       <c r="G49" t="n">
-        <v>274.7</v>
+        <v>44.7</v>
       </c>
       <c r="H49" t="n">
-        <v>871.1</v>
+        <v>196.3</v>
       </c>
       <c r="I49" t="n">
-        <v>871.1</v>
+        <v>255.5</v>
       </c>
     </row>
     <row r="50">
@@ -1920,25 +1920,25 @@
         <v>10</v>
       </c>
       <c r="C50" t="n">
-        <v>131.4</v>
+        <v>5</v>
       </c>
       <c r="D50" t="n">
-        <v>219.6</v>
+        <v>5.2</v>
       </c>
       <c r="E50" t="n">
-        <v>243</v>
+        <v>5.6</v>
       </c>
       <c r="F50" t="n">
-        <v>254.6</v>
+        <v>13.2</v>
       </c>
       <c r="G50" t="n">
-        <v>302.4</v>
+        <v>46.5</v>
       </c>
       <c r="H50" t="n">
-        <v>625.6</v>
+        <v>195.8</v>
       </c>
       <c r="I50" t="n">
-        <v>625.6</v>
+        <v>244.6</v>
       </c>
     </row>
     <row r="51">
@@ -1953,25 +1953,25 @@
         </is>
       </c>
       <c r="C51" s="2" t="n">
-        <v>148.43</v>
+        <v>4.99</v>
       </c>
       <c r="D51" s="2" t="n">
-        <v>209.29</v>
+        <v>5.15</v>
       </c>
       <c r="E51" s="2" t="n">
-        <v>239.12</v>
+        <v>5.42</v>
       </c>
       <c r="F51" s="2" t="n">
-        <v>258.53</v>
+        <v>10.47</v>
       </c>
       <c r="G51" s="2" t="n">
-        <v>291.52</v>
+        <v>44.97</v>
       </c>
       <c r="H51" s="2" t="n">
-        <v>633.99</v>
+        <v>197.18</v>
       </c>
       <c r="I51" s="2" t="n">
-        <v>633.99</v>
+        <v>262</v>
       </c>
     </row>
     <row r="52">
@@ -1986,25 +1986,25 @@
         </is>
       </c>
       <c r="C52" s="3" t="n">
-        <v>17.063</v>
+        <v>0.137</v>
       </c>
       <c r="D52" s="3" t="n">
-        <v>9.548999999999999</v>
+        <v>0.143</v>
       </c>
       <c r="E52" s="3" t="n">
-        <v>8.673</v>
+        <v>0.193</v>
       </c>
       <c r="F52" s="3" t="n">
-        <v>8.795999999999999</v>
+        <v>1.255</v>
       </c>
       <c r="G52" s="3" t="n">
-        <v>21.774</v>
+        <v>1.894</v>
       </c>
       <c r="H52" s="3" t="n">
-        <v>170.416</v>
+        <v>2.637</v>
       </c>
       <c r="I52" s="3" t="n">
-        <v>170.416</v>
+        <v>22.368</v>
       </c>
     </row>
   </sheetData>
@@ -2123,46 +2123,46 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>149.3</v>
+        <v>4.96</v>
       </c>
       <c r="C2" t="n">
-        <v>206.67</v>
+        <v>5.12</v>
       </c>
       <c r="D2" t="n">
-        <v>241.89</v>
+        <v>5.37</v>
       </c>
       <c r="E2" t="n">
-        <v>262.02</v>
+        <v>10.96</v>
       </c>
       <c r="F2" t="n">
-        <v>299.87</v>
+        <v>45.71</v>
       </c>
       <c r="G2" t="n">
-        <v>694.1799999999999</v>
+        <v>199.41</v>
       </c>
       <c r="H2" t="n">
-        <v>694.1799999999999</v>
+        <v>271.33</v>
       </c>
       <c r="I2" t="n">
-        <v>13.937</v>
+        <v>0.052</v>
       </c>
       <c r="J2" t="n">
-        <v>11.834</v>
+        <v>0.042</v>
       </c>
       <c r="K2" t="n">
-        <v>3.723</v>
+        <v>0.082</v>
       </c>
       <c r="L2" t="n">
-        <v>6.221</v>
+        <v>1.007</v>
       </c>
       <c r="M2" t="n">
-        <v>12.707</v>
+        <v>2.553</v>
       </c>
       <c r="N2" t="n">
-        <v>385.735</v>
+        <v>3.195</v>
       </c>
       <c r="O2" t="n">
-        <v>385.735</v>
+        <v>43.984</v>
       </c>
     </row>
     <row r="3">
@@ -2172,46 +2172,46 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>158.58</v>
+        <v>4.98</v>
       </c>
       <c r="C3" t="n">
-        <v>203.67</v>
+        <v>5.14</v>
       </c>
       <c r="D3" t="n">
-        <v>230.68</v>
+        <v>5.44</v>
       </c>
       <c r="E3" t="n">
-        <v>255.55</v>
+        <v>11.42</v>
       </c>
       <c r="F3" t="n">
-        <v>283.94</v>
+        <v>46.18</v>
       </c>
       <c r="G3" t="n">
-        <v>704.0700000000001</v>
+        <v>199.22</v>
       </c>
       <c r="H3" t="n">
-        <v>704.0700000000001</v>
+        <v>273</v>
       </c>
       <c r="I3" t="n">
-        <v>13.654</v>
+        <v>0.114</v>
       </c>
       <c r="J3" t="n">
-        <v>5.349</v>
+        <v>0.143</v>
       </c>
       <c r="K3" t="n">
-        <v>7.094</v>
+        <v>0.151</v>
       </c>
       <c r="L3" t="n">
-        <v>7.345</v>
+        <v>0.986</v>
       </c>
       <c r="M3" t="n">
-        <v>6.818</v>
+        <v>2.778</v>
       </c>
       <c r="N3" t="n">
-        <v>190.214</v>
+        <v>2.231</v>
       </c>
       <c r="O3" t="n">
-        <v>190.214</v>
+        <v>23.323</v>
       </c>
     </row>
     <row r="4">
@@ -2221,46 +2221,46 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>134.14</v>
+        <v>5.11</v>
       </c>
       <c r="C4" t="n">
-        <v>212.78</v>
+        <v>5.6</v>
       </c>
       <c r="D4" t="n">
-        <v>245.77</v>
+        <v>9.130000000000001</v>
       </c>
       <c r="E4" t="n">
-        <v>265.65</v>
+        <v>21.37</v>
       </c>
       <c r="F4" t="n">
-        <v>324.5</v>
+        <v>44.52</v>
       </c>
       <c r="G4" t="n">
-        <v>836.1900000000001</v>
+        <v>204.64</v>
       </c>
       <c r="H4" t="n">
-        <v>836.1900000000001</v>
+        <v>331.15</v>
       </c>
       <c r="I4" t="n">
-        <v>6.78</v>
+        <v>0.057</v>
       </c>
       <c r="J4" t="n">
-        <v>7.777</v>
+        <v>0.067</v>
       </c>
       <c r="K4" t="n">
-        <v>5.722</v>
+        <v>0.283</v>
       </c>
       <c r="L4" t="n">
-        <v>6.946</v>
+        <v>0.221</v>
       </c>
       <c r="M4" t="n">
-        <v>27.259</v>
+        <v>1.251</v>
       </c>
       <c r="N4" t="n">
-        <v>260.729</v>
+        <v>1.465</v>
       </c>
       <c r="O4" t="n">
-        <v>260.729</v>
+        <v>58.357</v>
       </c>
     </row>
     <row r="5">
@@ -2270,46 +2270,46 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>148.43</v>
+        <v>4.99</v>
       </c>
       <c r="C5" t="n">
-        <v>209.29</v>
+        <v>5.15</v>
       </c>
       <c r="D5" t="n">
-        <v>239.12</v>
+        <v>5.42</v>
       </c>
       <c r="E5" t="n">
-        <v>258.53</v>
+        <v>10.47</v>
       </c>
       <c r="F5" t="n">
-        <v>291.52</v>
+        <v>44.97</v>
       </c>
       <c r="G5" t="n">
-        <v>633.99</v>
+        <v>197.18</v>
       </c>
       <c r="H5" t="n">
-        <v>633.99</v>
+        <v>262</v>
       </c>
       <c r="I5" t="n">
-        <v>17.063</v>
+        <v>0.137</v>
       </c>
       <c r="J5" t="n">
-        <v>9.548999999999999</v>
+        <v>0.143</v>
       </c>
       <c r="K5" t="n">
-        <v>8.673</v>
+        <v>0.193</v>
       </c>
       <c r="L5" t="n">
-        <v>8.795999999999999</v>
+        <v>1.255</v>
       </c>
       <c r="M5" t="n">
-        <v>21.774</v>
+        <v>1.894</v>
       </c>
       <c r="N5" t="n">
-        <v>170.416</v>
+        <v>2.637</v>
       </c>
       <c r="O5" t="n">
-        <v>170.416</v>
+        <v>22.368</v>
       </c>
     </row>
   </sheetData>

</xml_diff>